<commit_message>
Added AAV Grant Form and updated MS Intro docx
</commit_message>
<xml_diff>
--- a/BBDetections.xlsx
+++ b/BBDetections.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kelseymccune/Documents/GitHub/BackyardBirds/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alex/Documents/GitHub/BackyardBirds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A6055D2-E8C3-E643-AAD1-AEF4DEC0FD9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3B82620-5A1A-BA44-8574-C934B1D0595B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18800" xr2:uid="{AFD5C794-3CDA-7B4E-95CA-1FB2B4E8F527}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{AFD5C794-3CDA-7B4E-95CA-1FB2B4E8F527}"/>
   </bookViews>
   <sheets>
     <sheet name="BBDetections" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10909" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10913" uniqueCount="201">
   <si>
     <t>Site</t>
   </si>
@@ -621,12 +621,15 @@
   <si>
     <t>16/09/2025</t>
   </si>
+  <si>
+    <t>29/09/2025</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -766,6 +769,25 @@
       <color rgb="FF000000"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1109,13 +1131,17 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="21" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="21" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1491,7 +1517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1F4F9FE-882E-E541-B783-9FA7CCC4A27B}">
-  <dimension ref="A1:H2950"/>
+  <dimension ref="A1:I2953"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -69218,7 +69244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2945" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2945" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2945" t="s">
         <v>31</v>
       </c>
@@ -69241,7 +69267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2946" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2946" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2946" t="s">
         <v>31</v>
       </c>
@@ -69264,7 +69290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2947" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2947" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2947" t="s">
         <v>31</v>
       </c>
@@ -69287,7 +69313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2948" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2948" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2948" t="s">
         <v>31</v>
       </c>
@@ -69310,7 +69336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2949" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2949" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2949" t="s">
         <v>31</v>
       </c>
@@ -69333,7 +69359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2950" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2950" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2950" t="s">
         <v>31</v>
       </c>
@@ -69355,6 +69381,52 @@
       <c r="G2950" s="3">
         <v>1</v>
       </c>
+    </row>
+    <row r="2951" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2951" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2951" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2951" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2951" s="7">
+        <v>28.9</v>
+      </c>
+      <c r="E2951" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="F2951" s="8">
+        <v>0.6997916666666667</v>
+      </c>
+      <c r="G2951" s="7">
+        <v>1</v>
+      </c>
+      <c r="H2951" s="7"/>
+      <c r="I2951" s="6"/>
+    </row>
+    <row r="2952" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2952" s="7"/>
+      <c r="B2952" s="7"/>
+      <c r="C2952" s="7"/>
+      <c r="D2952" s="7"/>
+      <c r="E2952" s="7"/>
+      <c r="F2952" s="7"/>
+      <c r="G2952" s="7"/>
+      <c r="H2952" s="7"/>
+      <c r="I2952" s="6"/>
+    </row>
+    <row r="2953" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2953" s="9"/>
+      <c r="B2953" s="9"/>
+      <c r="C2953" s="9"/>
+      <c r="D2953" s="9"/>
+      <c r="E2953" s="9"/>
+      <c r="F2953" s="9"/>
+      <c r="G2953" s="9"/>
+      <c r="H2953" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>